<commit_message>
Update crop acreage breakdown: 1,600 corn / 700 hay / 200 wheat-rye, replacing incorrect Soybeans row
</commit_message>
<xml_diff>
--- a/data/Crop Detail by Field - Type.xlsx
+++ b/data/Crop Detail by Field - Type.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -472,6 +472,9 @@
           <t>Corn Silage</t>
         </is>
       </c>
+      <c r="B2" t="n">
+        <v>1600</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -479,12 +482,18 @@
           <t>Alfalfa Hay</t>
         </is>
       </c>
+      <c r="B3" t="n">
+        <v>700</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Soybeans</t>
-        </is>
+          <t>Wheat/Rye</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>200</v>
       </c>
     </row>
     <row r="5">

</xml_diff>